<commit_message>
feat: verify rule CG0131 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000006/negative/01/data/unit-test-coreid-CG0131-negative.xlsx
+++ b/rules/CORE-000006/negative/01/data/unit-test-coreid-CG0131-negative.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="dm.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dm.xpt" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,6 +608,90 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DTHFL</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DTHFL</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DTHFL</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -681,7 +765,7 @@
           <t>DTHDTC</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>DTHFL</t>
         </is>

</xml_diff>